<commit_message>
messages bug fix and encryption
</commit_message>
<xml_diff>
--- a/docs/CareerCraft_Test_Cases.xlsx
+++ b/docs/CareerCraft_Test_Cases.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B12EAC-865E-47F6-9966-125386DC03B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{270FC3ED-1E95-4BAA-96C3-6912F8284D71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="222">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -64,6 +64,9 @@
     <t>User is successfully registered and redirected to Dashboard</t>
   </si>
   <si>
+    <t>Pass</t>
+  </si>
+  <si>
     <t>TC-002</t>
   </si>
   <si>
@@ -336,14 +339,381 @@
     <t>Course is drafted and available for curriculum editing</t>
   </si>
   <si>
-    <t>Pass</t>
+    <t>TC-016</t>
+  </si>
+  <si>
+    <t>Live Coding</t>
+  </si>
+  <si>
+    <t>LiveKit Connection</t>
+  </si>
+  <si>
+    <t>Verify LiveKit room connects successfully when starting interview</t>
+  </si>
+  <si>
+    <t>Navigated to active interview page</t>
+  </si>
+  <si>
+    <t>1. Click Start Interview</t>
+  </si>
+  <si>
+    <t>Connected to LiveKit room and VAPI agent successfully</t>
+  </si>
+  <si>
+    <t>TC-017</t>
+  </si>
+  <si>
+    <t>LiveKit Code Share</t>
+  </si>
+  <si>
+    <t>Verify code editor changes are shared to VAPI agent in real-time via LiveKit</t>
+  </si>
+  <si>
+    <t>In active Live Coding Interview</t>
+  </si>
+  <si>
+    <t>1. Type code in monaco editor</t>
+  </si>
+  <si>
+    <t>VAPI agent receives updated code context and responds accordingly</t>
+  </si>
+  <si>
+    <t>TC-018</t>
+  </si>
+  <si>
+    <t>LiveKit Disconnect</t>
+  </si>
+  <si>
+    <t>Verify LiveKit room disconnects on interview end</t>
+  </si>
+  <si>
+    <t>In active interview</t>
+  </si>
+  <si>
+    <t>1. Click End Interview</t>
+  </si>
+  <si>
+    <t>LiveKit room connection is closed securely</t>
+  </si>
+  <si>
+    <t>TC-019</t>
+  </si>
+  <si>
+    <t>Social Media</t>
+  </si>
+  <si>
+    <t>Direct Messaging</t>
+  </si>
+  <si>
+    <t>Verify user can send a direct message to a friend</t>
+  </si>
+  <si>
+    <t>Logged in, on friend chat page</t>
+  </si>
+  <si>
+    <t>1. Type message
+2. Click Send</t>
+  </si>
+  <si>
+    <t>Message appears in chat history and is stored in Firestore</t>
+  </si>
+  <si>
+    <t>TC-020</t>
+  </si>
+  <si>
+    <t>Receive Message</t>
+  </si>
+  <si>
+    <t>Verify user receives message in real-time</t>
+  </si>
+  <si>
+    <t>Both users on chat page</t>
+  </si>
+  <si>
+    <t>1. Friend sends a message</t>
+  </si>
+  <si>
+    <t>Message appears instantly without refreshing the page</t>
+  </si>
+  <si>
+    <t>TC-021</t>
+  </si>
+  <si>
+    <t>Chat History</t>
+  </si>
+  <si>
+    <t>Verify chat history loads when opening chat</t>
+  </si>
+  <si>
+    <t>Previous messages exist</t>
+  </si>
+  <si>
+    <t>1. Open chat with friend</t>
+  </si>
+  <si>
+    <t>Previous messages are displayed correctly in order</t>
+  </si>
+  <si>
+    <t>TC-022</t>
+  </si>
+  <si>
+    <t>Failed Payment</t>
+  </si>
+  <si>
+    <t>Verify failed payment handles gracefully</t>
+  </si>
+  <si>
+    <t>On payment gateway</t>
+  </si>
+  <si>
+    <t>1. Enter invalid card details
+2. Submit</t>
+  </si>
+  <si>
+    <t>Error message displayed, course remains locked</t>
+  </si>
+  <si>
+    <t>TC-023</t>
+  </si>
+  <si>
+    <t>Course Unlocking</t>
+  </si>
+  <si>
+    <t>Verify course unlocks immediately after successful payment</t>
+  </si>
+  <si>
+    <t>Course is locked, payment completed</t>
+  </si>
+  <si>
+    <t>1. Navigate to course page</t>
+  </si>
+  <si>
+    <t>Course content is accessible without requiring manual refresh</t>
+  </si>
+  <si>
+    <t>TC-024</t>
+  </si>
+  <si>
+    <t>Webhook Processing</t>
+  </si>
+  <si>
+    <t>Verify backend updates database on payment success</t>
+  </si>
+  <si>
+    <t>Payment completed</t>
+  </si>
+  <si>
+    <t>1. Check user enrollment in Firestore</t>
+  </si>
+  <si>
+    <t>User document has new course ID in enrolled array</t>
+  </si>
+  <si>
+    <t>TC-025</t>
+  </si>
+  <si>
+    <t>Payment History</t>
+  </si>
+  <si>
+    <t>Verify user can view their past transactions</t>
+  </si>
+  <si>
+    <t>User has made purchases</t>
+  </si>
+  <si>
+    <t>1. Go to Profile -&gt; Billing/Payments</t>
+  </si>
+  <si>
+    <t>List of successful transactions is displayed</t>
+  </si>
+  <si>
+    <t>TC-026</t>
+  </si>
+  <si>
+    <t>Contact Us</t>
+  </si>
+  <si>
+    <t>Form Submission</t>
+  </si>
+  <si>
+    <t>Verify form submits with valid data</t>
+  </si>
+  <si>
+    <t>On Contact Us page</t>
+  </si>
+  <si>
+    <t>1. Fill name, email, message
+2. Click Submit</t>
+  </si>
+  <si>
+    <t>Success message shown, email sent via nodemailer/API</t>
+  </si>
+  <si>
+    <t>TC-027</t>
+  </si>
+  <si>
+    <t>Form Validation</t>
+  </si>
+  <si>
+    <t>Verify form requires all fields</t>
+  </si>
+  <si>
+    <t>1. Leave fields blank
+2. Click Submit</t>
+  </si>
+  <si>
+    <t>Validation errors displayed for required fields</t>
+  </si>
+  <si>
+    <t>TC-028</t>
+  </si>
+  <si>
+    <t>Email Validation</t>
+  </si>
+  <si>
+    <t>Verify email field checks format</t>
+  </si>
+  <si>
+    <t>1. Enter invalid email (e.g. 'test@')
+2. Click Submit</t>
+  </si>
+  <si>
+    <t>Error message 'Invalid email address'</t>
+  </si>
+  <si>
+    <t>TC-029</t>
+  </si>
+  <si>
+    <t>Loading State</t>
+  </si>
+  <si>
+    <t>Verify submit button shows loading state</t>
+  </si>
+  <si>
+    <t>Form filled correctly</t>
+  </si>
+  <si>
+    <t>1. Click Submit</t>
+  </si>
+  <si>
+    <t>Button disables and shows a spinner while sending</t>
+  </si>
+  <si>
+    <t>TC-030</t>
+  </si>
+  <si>
+    <t>Chat Bot</t>
+  </si>
+  <si>
+    <t>Open Bot</t>
+  </si>
+  <si>
+    <t>Verify clicking bot icon opens chat window</t>
+  </si>
+  <si>
+    <t>Logged in</t>
+  </si>
+  <si>
+    <t>1. Click Chat Bot floating icon</t>
+  </si>
+  <si>
+    <t>Chat Bot window expands and shows greeting</t>
+  </si>
+  <si>
+    <t>TC-031</t>
+  </si>
+  <si>
+    <t>Text Response</t>
+  </si>
+  <si>
+    <t>Verify bot responds to text input</t>
+  </si>
+  <si>
+    <t>Chat Bot open</t>
+  </si>
+  <si>
+    <t>1. Type 'Hello'
+2. Send</t>
+  </si>
+  <si>
+    <t>Bot replies with an appropriate greeting</t>
+  </si>
+  <si>
+    <t>TC-032</t>
+  </si>
+  <si>
+    <t>Voice Input (Vapi)</t>
+  </si>
+  <si>
+    <t>Verify voice interaction works</t>
+  </si>
+  <si>
+    <t>Chat Bot open, microphone allowed</t>
+  </si>
+  <si>
+    <t>1. Click microphone
+2. Speak to bot
+3. Stop</t>
+  </si>
+  <si>
+    <t>Bot processes speech and responds with audio/text</t>
+  </si>
+  <si>
+    <t>TC-033</t>
+  </si>
+  <si>
+    <t>Career Advice Context</t>
+  </si>
+  <si>
+    <t>Verify bot gives relevant career advice</t>
+  </si>
+  <si>
+    <t>1. Ask 'How to become a frontend dev?'</t>
+  </si>
+  <si>
+    <t>Bot provides a structured, relevant career guide</t>
+  </si>
+  <si>
+    <t>TC-034</t>
+  </si>
+  <si>
+    <t>Network Disconnect</t>
+  </si>
+  <si>
+    <t>Verify bot handles network disconnects</t>
+  </si>
+  <si>
+    <t>1. Disconnect internet
+2. Send message</t>
+  </si>
+  <si>
+    <t>Error message indicating offline status</t>
+  </si>
+  <si>
+    <t>TC-035</t>
+  </si>
+  <si>
+    <t>Session Persistence</t>
+  </si>
+  <si>
+    <t>Verify chat history persists during session</t>
+  </si>
+  <si>
+    <t>Have previous messages in bot</t>
+  </si>
+  <si>
+    <t>1. Close bot
+2. Reopen bot</t>
+  </si>
+  <si>
+    <t>Previous messages from the session are still visible</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -353,7 +723,13 @@
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FF008000"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -370,7 +746,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -378,20 +754,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -732,52 +1126,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="35" customWidth="1"/>
-    <col min="5" max="5" width="25" customWidth="1"/>
-    <col min="6" max="6" width="45" customWidth="1"/>
-    <col min="7" max="7" width="35" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="7" width="40" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -792,372 +1185,892 @@
       <c r="G2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>101</v>
+      <c r="H2" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="2" t="s">
+      <c r="A3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>16</v>
+      <c r="C3" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>101</v>
+        <v>21</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>23</v>
       </c>
+      <c r="C4" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="D4" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="F12" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>79</v>
+      <c r="C13" s="3" t="s">
+        <v>80</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>101</v>
+        <v>84</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>85</v>
       </c>
+      <c r="B14" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>86</v>
+      </c>
       <c r="D14" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>12</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>101</v>
+        <v>89</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>90</v>
       </c>
+      <c r="B15" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="D15" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>12</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="H15" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G16" s="3" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>101</v>
+      <c r="H16" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A33" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>